<commit_message>
Refactor employee mobile pages to use new MobileShell and WalletHero components; enhance home model creation for regular and flexible employees; update styles and structure for better responsiveness and usability.
</commit_message>
<xml_diff>
--- a/backend/templates/sao_ke_tt_theo_du_an.xlsx
+++ b/backend/templates/sao_ke_tt_theo_du_an.xlsx
@@ -710,26 +710,26 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>257175</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>219075</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D73BDFEA-77F9-846B-04BC-DD2B076F2AE1}"/>
+              <a16:creationId id="{D73BDFEA-77F9-846B-04BC-DD2B076F2AE1}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -738,15 +738,15 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:blip r:embed="rId1"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="257175" y="2133600"/>
-          <a:ext cx="476250" cy="476250"/>
+          <a:off x="0" y="1714500"/>
+          <a:ext cx="2743200" cy="1097280"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -773,10 +773,10 @@
         <xdr:cNvPr id="4" name="Picture 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4BED79A2-C0BF-5BD4-876D-5F228E845E0C}"/>
+              <a16:creationId id="{4BED79A2-C0BF-5BD4-876D-5F228E845E0C}"/>
             </a:ext>
             <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
-              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{D73BDFEA-77F9-846B-04BC-DD2B076F2AE1}"/>
+              <a16:predDERef pred="{D73BDFEA-77F9-846B-04BC-DD2B076F2AE1}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -785,7 +785,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:blip r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1077,7 +1077,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -1156,9 +1156,7 @@
     </row>
     <row r="7" spans="1:5" ht="22.5" customHeight="1">
       <c r="A7" s="3"/>
-      <c r="B7" s="36" t="s">
-        <v>10</v>
-      </c>
+      <c r="B7" s="36"/>
       <c r="C7" s="36"/>
       <c r="D7" s="37" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
feat: add FlexPay reconciliation exporter tests and improve Excel generation
- Implement tests for FlexPay reconciliation exporter to ensure no orphaned table relationships, contiguous worksheet parts, and undeclared ignorable prefixes in generated Excel files.
- Enhance Payroll report exporter to remove template tables and sanitize workbook XML before returning the final Excel bytes.
- Update various dialog components across the frontend to standardize padding and improve layout consistency.
- Refactor dialog content components to accept a new `contentPadding` prop for better control over padding behavior.
</commit_message>
<xml_diff>
--- a/backend/templates/sao_ke_tt_theo_du_an.xlsx
+++ b/backend/templates/sao_ke_tt_theo_du_an.xlsx
@@ -803,21 +803,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{68E53EB8-FD1A-4AA9-9E81-1495ABEA4FCE}" name="Table1" displayName="Table1" ref="A8:F12" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8" headerRowBorderDxfId="6" tableBorderDxfId="7" totalsRowBorderDxfId="5">
-  <autoFilter ref="A8:F12" xr:uid="{68E53EB8-FD1A-4AA9-9E81-1495ABEA4FCE}"/>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{4D1C5451-8DAC-4C0C-A2F5-7732B47DEA04}" name="STT" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{B79BC3B4-3AFD-4BA3-86C9-2386AFCD2550}" name="Họ tên" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{F8BDC4AC-E99E-4DE2-872F-38DA43D8AB6F}" name="CCCD" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{E4623EC1-2C6E-416E-B0FC-E1D9C4F516AA}" name="Dự án" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{75190708-1BC8-46D5-8C71-E3A86E561AD7}" name="Số tiền"/>
-    <tableColumn id="5" xr3:uid="{9B07B4F5-CE3F-4731-AD0B-CD60D14F13E7}" name="Ngày trả" dataDxfId="0"/>
-  </tableColumns>
-  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1466,8 +1451,5 @@
     <mergeCell ref="A4:B4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>